<commit_message>
Feature de Fondos, refactors de backend y actualización de datos
- Nueva funcionalidad de Fondos (backend: routes/funds.py, fund_service.py;
  frontend: página Funds, gráficos de saldo/flatten, ledger enriquecido)
- Refactors y mejoras en servicios de sources, transactions, dashboard,
  variables y storage; ajustes en Debts, DataExplorer, Sources y api.ts
- Datos actualizados (etiquetado, interpolaciones, procesada) y nuevos
  archivos de origen en data/nuevos
- Datos mock (data_mock) y scripts de generación/depuración
- Pruebas nuevas (tests de rutas y de tarjetas)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/sistema/procesada/tarjeta/tarjeta_metadata_unida.xlsx
+++ b/data/sistema/procesada/tarjeta/tarjeta_metadata_unida.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q27"/>
+  <dimension ref="A1:Q31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2013,19 +2013,19 @@
         <v>227.69</v>
       </c>
       <c r="J27" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="K27" s="1" t="n">
         <v>46058</v>
       </c>
       <c r="L27" s="1" t="n">
-        <v>46080</v>
+        <v>46087</v>
       </c>
       <c r="M27" t="n">
-        <v>229.65</v>
+        <v>230.32</v>
       </c>
       <c r="N27" t="n">
-        <v>459.97</v>
+        <v>460.64</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -2033,9 +2033,237 @@
         </is>
       </c>
       <c r="P27" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>BANCO PICHINCHA</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>3067XXXXXX5647</t>
+        </is>
+      </c>
+      <c r="C28" s="1" t="n">
+        <v>46118</v>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="n">
+        <v>230.32</v>
+      </c>
+      <c r="F28" t="n">
         <v>0</v>
       </c>
-      <c r="Q27" t="b">
+      <c r="G28" t="n">
+        <v>442.61</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" t="n">
+        <v>439.98</v>
+      </c>
+      <c r="J28" t="n">
+        <v>26</v>
+      </c>
+      <c r="K28" s="1" t="n">
+        <v>46088</v>
+      </c>
+      <c r="L28" s="1" t="n">
+        <v>46113</v>
+      </c>
+      <c r="M28" t="n">
+        <v>442.61</v>
+      </c>
+      <c r="N28" t="n">
+        <v>885.22</v>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Abril26.pdf</t>
+        </is>
+      </c>
+      <c r="P28" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q28" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>BANCO PICHINCHA</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>3067XXXXXX5647</t>
+        </is>
+      </c>
+      <c r="C29" s="1" t="n">
+        <v>46148</v>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="n">
+        <v>442.61</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" t="n">
+        <v>860.92</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" t="n">
+        <v>431.23</v>
+      </c>
+      <c r="J29" t="n">
+        <v>22</v>
+      </c>
+      <c r="K29" s="1" t="n">
+        <v>46116</v>
+      </c>
+      <c r="L29" s="1" t="n">
+        <v>46148</v>
+      </c>
+      <c r="M29" t="n">
+        <v>438.3100000000001</v>
+      </c>
+      <c r="N29" t="n">
+        <v>1299.23</v>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>Mayo26.pdf</t>
+        </is>
+      </c>
+      <c r="P29" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q29" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>BANCO PICHINCHA</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>3067XXXXXX5647</t>
+        </is>
+      </c>
+      <c r="C30" s="1" t="n">
+        <v>46179</v>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="n">
+        <v>860.92</v>
+      </c>
+      <c r="F30" t="n">
+        <v>860.92</v>
+      </c>
+      <c r="G30" t="n">
+        <v>266.96</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" t="n">
+        <v>254.3</v>
+      </c>
+      <c r="J30" t="n">
+        <v>31</v>
+      </c>
+      <c r="K30" s="1" t="n">
+        <v>46148</v>
+      </c>
+      <c r="L30" s="1" t="n">
+        <v>46179</v>
+      </c>
+      <c r="M30" t="n">
+        <v>266.96</v>
+      </c>
+      <c r="N30" t="n">
+        <v>533.92</v>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>Junio26.pdf</t>
+        </is>
+      </c>
+      <c r="P30" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q30" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>BANCO PICHINCHA</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>3067XXXXXX5647</t>
+        </is>
+      </c>
+      <c r="C31" s="1" t="n">
+        <v>46209</v>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="n">
+        <v>266.96</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" t="n">
+        <v>199.74</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" t="n">
+        <v>190.1</v>
+      </c>
+      <c r="J31" t="n">
+        <v>32</v>
+      </c>
+      <c r="K31" s="1" t="n">
+        <v>46182</v>
+      </c>
+      <c r="L31" s="1" t="n">
+        <v>46207</v>
+      </c>
+      <c r="M31" t="n">
+        <v>199.74</v>
+      </c>
+      <c r="N31" t="n">
+        <v>399.48</v>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>Julio26.pdf</t>
+        </is>
+      </c>
+      <c r="P31" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q31" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>